<commit_message>
feat(lighthab): finish carrier migration
</commit_message>
<xml_diff>
--- a/outputs/fit-check-order-list.xlsx
+++ b/outputs/fit-check-order-list.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re5a6217d0f224899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order List" sheetId="2" r:id="R3a7eb7a873a44e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hold Closure" sheetId="3" r:id="R1d5fb0a124114eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1638369846bf4564"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order List" sheetId="2" r:id="R3a8c42fd0a8d46d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hold Closure" sheetId="3" r:id="Re447713810184260"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,8 +212,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FitCheckOrderTable" displayName="FitCheckOrderTable" ref="A1:J34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FitCheckOrderTable" displayName="FitCheckOrderTable" ref="A1:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J23"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Category"/>
@@ -231,7 +231,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HoldClosureTable" displayName="HoldClosureTable" ref="A1:D7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HoldClosureTable" displayName="HoldClosureTable" ref="A1:D9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Held item"/>
     <x:tableColumn id="2" name="Reason"/>
@@ -460,7 +460,7 @@
         <x:v>Prepared</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>2026-09-20</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -476,8 +476,8 @@
         <x:v>Buy-now line items</x:v>
       </x:c>
       <x:c r="B5" s="9" t="n">
-        <x:f>COUNTIF('Order List'!$A$2:$A$34,"BUY NOW")</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTIF('Order List'!$A$2:$A$23,"BUY NOW")</x:f>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -485,8 +485,8 @@
         <x:v>Held line items</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:f>COUNTIF('Order List'!$A$2:$A$34,"HOLD")</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIF('Order List'!$A$2:$A$23,"HOLD")</x:f>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -494,7 +494,7 @@
         <x:v>Required populated PCB refs</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:v>23</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -535,10 +535,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Use pre-crimp leads</x:v>
+        <x:v>Measure LightHAB first</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>Avoids specialized JST production tooling for the prototype.</x:v>
+        <x:v>J1/J2/J3 and all four mounting holes remain provisional until the purchased tracker is measured.</x:v>
       </x:c>
       <x:c r="D12" s="12"/>
       <x:c r="E12" s="12"/>
@@ -549,10 +549,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>Observe J1 limit</x:v>
+        <x:v>Use pre-crimp J5 leads</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>JST-PH is at the 2 A cutdown-current edge; pulse/cold test the finished harness.</x:v>
+        <x:v>Avoids specialized JST production tooling for the prototype cutdown harness.</x:v>
       </x:c>
       <x:c r="D13" s="12"/>
       <x:c r="E13" s="12"/>
@@ -566,7 +566,7 @@
         <x:v>Keep flight-critical holds</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>Antenna, LPF, nichrome, sleeves, and final spacers need physical/test inputs.</x:v>
+        <x:v>Interfaces, antennas, nichrome, sleeves, and final spacers need physical or test inputs.</x:v>
       </x:c>
       <x:c r="D14" s="12"/>
       <x:c r="E14" s="12"/>
@@ -707,7 +707,7 @@
         <x:v>Use included straight header</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="60" hidden="0" customHeight="1">
+    <x:row r="4" ht="84" hidden="0" customHeight="1">
       <x:c r="A4" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
@@ -718,10 +718,10 @@
         <x:v>Host</x:v>
       </x:c>
       <x:c r="D4" s="19" t="str">
-        <x:v>LightAPRS-W 2.0 (+WSPR)</x:v>
+        <x:v>LightHABTracker 1.0</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>GPS/APRS/WSPR host module</x:v>
+        <x:v>GPS/APRS/WSPR tracker with 3xAA holder and two pyro outputs</x:v>
       </x:c>
       <x:c r="F4" s="20" t="n">
         <x:v>1</x:v>
@@ -733,10 +733,10 @@
         <x:v>QRP Labs</x:v>
       </x:c>
       <x:c r="I4" s="19" t="str">
-        <x:v>https://www.qrp-labs.com/lightaprsw2.html</x:v>
+        <x:v>https://shop.qrp-labs.com/aprs/LightHABTracker</x:v>
       </x:c>
       <x:c r="J4" s="19" t="str">
-        <x:v>Exact 2.0 WSPR-capable module</x:v>
+        <x:v>Measure the purchased board before fabricating the carrier</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="96" hidden="0" customHeight="1">
@@ -747,7 +747,7 @@
         <x:v>Capacitor</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>C1,C5</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
         <x:v>C322C475K5R5TA</x:v>
@@ -756,10 +756,10 @@
         <x:v>4.7 uF radial THT capacitor</x:v>
       </x:c>
       <x:c r="F5" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="20" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H5" s="19" t="str">
         <x:v>DigiKey</x:v>
@@ -779,7 +779,7 @@
         <x:v>Capacitor</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>C2-C4</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
         <x:v>C315C104K5R5TA</x:v>
@@ -788,10 +788,10 @@
         <x:v>0.1 uF radial THT capacitor</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="20" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H6" s="19" t="str">
         <x:v>DigiKey</x:v>
@@ -833,7 +833,7 @@
       </x:c>
       <x:c r="J7" s="19" t="str"/>
     </x:row>
-    <x:row r="8" ht="120" hidden="0" customHeight="1">
+    <x:row r="8" ht="108" hidden="0" customHeight="1">
       <x:c r="A8" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
@@ -841,13 +841,13 @@
         <x:v>PCB connector</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
-        <x:v>J1</x:v>
+        <x:v>J5</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
-        <x:v>S2B-PH-K-S(LF)(SN)</x:v>
+        <x:v>S2B-XH-A(LF)(SN)</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>JST PH 2-pin side-entry THT header</x:v>
+        <x:v>JST XH 2-pin side-entry THT header</x:v>
       </x:c>
       <x:c r="F8" s="20" t="n">
         <x:v>1</x:v>
@@ -859,91 +859,89 @@
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I8" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=S2B-PH-K-S%28LF%29%28SN%29</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=S2B-XH-A%28LF%29%28SN%29</x:v>
       </x:c>
       <x:c r="J8" s="19" t="str">
-        <x:v>Battery input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="84" hidden="0" customHeight="1">
+        <x:v>Cutdown output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="96" hidden="0" customHeight="1">
       <x:c r="A9" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B9" s="19" t="str">
-        <x:v>Module header</x:v>
+        <x:v>Resistor</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
-        <x:v>J2</x:v>
+        <x:v>R1,R4</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>61301111121</x:v>
+        <x:v>MFR-25FBF52-1K</x:v>
       </x:c>
       <x:c r="E9" s="19" t="str">
-        <x:v>1x11 2.54 mm straight THT header</x:v>
+        <x:v>1 kohm 1% 1/4 W axial</x:v>
       </x:c>
       <x:c r="F9" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H9" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I9" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=61301111121</x:v>
-      </x:c>
-      <x:c r="J9" s="19" t="str">
-        <x:v>LightAPRS edge interface</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="84" hidden="0" customHeight="1">
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-1K/13011</x:v>
+      </x:c>
+      <x:c r="J9" s="19" t="str"/>
+    </x:row>
+    <x:row r="10" ht="96" hidden="0" customHeight="1">
       <x:c r="A10" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B10" s="19" t="str">
-        <x:v>RF connector</x:v>
+        <x:v>Resistor</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
-        <x:v>J3,J4</x:v>
+        <x:v>R2</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>132134</x:v>
+        <x:v>MFR-25FBF52-100K</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>50-ohm standard SMA female THT jack</x:v>
+        <x:v>100 kohm 1% 1/4 W axial</x:v>
       </x:c>
       <x:c r="F10" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H10" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I10" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=132134</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=MFR-25FBF52-100K</x:v>
       </x:c>
       <x:c r="J10" s="19" t="str">
-        <x:v>Not RP-SMA</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="108" hidden="0" customHeight="1">
+        <x:v>LED reset-default-off pull-up</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="84" hidden="0" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B11" s="19" t="str">
-        <x:v>PCB connector</x:v>
+        <x:v>Cutdown harness</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>J5</x:v>
+        <x:v>J5 mate</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>S2B-XH-A(LF)(SN)</x:v>
+        <x:v>XHP-2</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>JST XH 2-pin side-entry THT header</x:v>
+        <x:v>JST XH 2-position receptacle housing</x:v>
       </x:c>
       <x:c r="F11" s="20" t="n">
         <x:v>1</x:v>
@@ -955,730 +953,386 @@
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I11" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=S2B-XH-A%28LF%29%28SN%29</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=XHP-2</x:v>
       </x:c>
       <x:c r="J11" s="19" t="str">
-        <x:v>Cutdown output</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="84" hidden="0" customHeight="1">
+        <x:v>Housing only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="120" hidden="0" customHeight="1">
       <x:c r="A12" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>RF/module pin</x:v>
+        <x:v>Cutdown harness</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>J6,J7</x:v>
+        <x:v>J5 leads</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>61300111121</x:v>
+        <x:v>ASXHSXH22K152</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>Single-pin 2.54 mm straight THT header</x:v>
+        <x:v>22 AWG 6-inch pre-crimp socket-to-socket lead</x:v>
       </x:c>
       <x:c r="F12" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G12" s="20" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=61300111121</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/jst-sales-america-inc/ASXHSXH22K152/6684931</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>LightAPRS VHF/HF contacts</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="84" hidden="0" customHeight="1">
+        <x:v>Cut in half; identify PACK+ and FET-</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" hidden="0" customHeight="1">
       <x:c r="A13" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
-        <x:v>MOSFET</x:v>
+        <x:v>Power</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:v>Q1</x:v>
+        <x:v>Flight/test cells</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
-        <x:v>IRLZ44NPBF</x:v>
+        <x:v>Energizer L91</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>Logic-level N-MOSFET, TO-220</x:v>
+        <x:v>AA lithium primary cell</x:v>
       </x:c>
       <x:c r="F13" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G13" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>Authorized retailer</x:v>
       </x:c>
       <x:c r="I13" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=IRLZ44NPBF</x:v>
-      </x:c>
-      <x:c r="J13" s="19" t="str"/>
-    </x:row>
-    <x:row r="14" ht="96" hidden="0" customHeight="1">
+        <x:v>https://data.energizer.com/pdfs/l91.pdf</x:v>
+      </x:c>
+      <x:c r="J13" s="19" t="str">
+        <x:v>Two matched 3-cell sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="84" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>Resistor</x:v>
+        <x:v>Storage</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>R1,R4</x:v>
+        <x:v>OpenLog media</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>MFR-25FBF52-1K</x:v>
+        <x:v>microSDHC &lt;=32 GB</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>1 kohm 1% 1/4 W axial</x:v>
+        <x:v>FAT32 microSD card</x:v>
       </x:c>
       <x:c r="F14" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G14" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G14" s="20" t="n">
-        <x:v>10</x:v>
-      </x:c>
       <x:c r="H14" s="19" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>Reputable retailer</x:v>
       </x:c>
       <x:c r="I14" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-1K/13011</x:v>
-      </x:c>
-      <x:c r="J14" s="19" t="str"/>
-    </x:row>
-    <x:row r="15" ht="96" hidden="0" customHeight="1">
+        <x:v>https://www.sparkfun.com/sparkfun-openlog-with-headers.html</x:v>
+      </x:c>
+      <x:c r="J14" s="19" t="str">
+        <x:v>One spare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="60" hidden="0" customHeight="1">
       <x:c r="A15" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B15" s="19" t="str">
-        <x:v>Resistor</x:v>
+        <x:v>Mechanical fit tool</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:v>R2</x:v>
+        <x:v>Module spacing</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
-        <x:v>MFR-25FBF52-100R</x:v>
+        <x:v>M2/M2.5 nylon hardware assortment</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>100 ohm 1% 1/4 W axial</x:v>
+        <x:v>Spacers, screws, and nuts</x:v>
       </x:c>
       <x:c r="F15" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G15" s="20" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I15" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=MFR-25FBF52-100R</x:v>
-      </x:c>
-      <x:c r="J15" s="19" t="str"/>
-    </x:row>
-    <x:row r="16" ht="96" hidden="0" customHeight="1">
+        <x:v>Local supplier</x:v>
+      </x:c>
+      <x:c r="I15" s="19" t="str"/>
+      <x:c r="J15" s="19" t="str">
+        <x:v>Fit tool only; final diameter and height held</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="84" hidden="0" customHeight="1">
       <x:c r="A16" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B16" s="19" t="str">
-        <x:v>Resistor</x:v>
+        <x:v>Module interface</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>R3</x:v>
+        <x:v>J1</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
-        <x:v>MFR-25FBF52-1M</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>1 Mohm 1% 1/4 W axial</x:v>
+        <x:v>Two-position VBATT/GND solder interface</x:v>
       </x:c>
       <x:c r="F16" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="20" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I16" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=MFR-25FBF52-1M</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I16" s="19" t="str"/>
       <x:c r="J16" s="19" t="str">
-        <x:v>Stock hold observed 2026-09-20; verify body before substitute</x:v>
+        <x:v>Measure pad pitch, hole size, and mating method on LightHAB</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="96" hidden="0" customHeight="1">
       <x:c r="A17" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B17" s="19" t="str">
-        <x:v>Switch</x:v>
+        <x:v>Module interface</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
-        <x:v>SW1</x:v>
+        <x:v>J2</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
-        <x:v>7101SYZQE</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>C&amp;K SPDT toggle, solder terminals</x:v>
+        <x:v>Nine-position signal solder interface</x:v>
       </x:c>
       <x:c r="F17" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I17" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/c-k/SWITCH-7101SYZQE/25966</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I17" s="19" t="str"/>
       <x:c r="J17" s="19" t="str">
-        <x:v>Do not substitute SYWQE</x:v>
+        <x:v>Verify actual row pitch, location, and installed header direction</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="84" hidden="0" customHeight="1">
       <x:c r="A18" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
-        <x:v>IC</x:v>
+        <x:v>Module interface</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
-        <x:v>U1</x:v>
+        <x:v>J3</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
-        <x:v>PCF8574N</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E18" s="19" t="str">
-        <x:v>I2C I/O expander, PDIP-16</x:v>
+        <x:v>Two-position OUT1/GND solder interface</x:v>
       </x:c>
       <x:c r="F18" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="19" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I18" s="19" t="str"/>
+      <x:c r="J18" s="19" t="str">
+        <x:v>Measure pad pitch, hole size, and mating method on LightHAB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" hidden="0" customHeight="1">
+      <x:c r="A19" s="19" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="str">
+        <x:v>Fabrication</x:v>
+      </x:c>
+      <x:c r="C19" s="19" t="str">
+        <x:v>Carrier PCB</x:v>
+      </x:c>
+      <x:c r="D19" s="19" t="str">
+        <x:v>Bare PCB</x:v>
+      </x:c>
+      <x:c r="E19" s="19" t="str">
+        <x:v>Fabricated weather-balloon-logger carrier</x:v>
+      </x:c>
+      <x:c r="F19" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G19" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="19" t="str">
+        <x:v>PCB fabricator</x:v>
+      </x:c>
+      <x:c r="I19" s="19" t="str"/>
+      <x:c r="J19" s="19" t="str">
+        <x:v>Order only after exact-parts 1:1 fit gate passes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="108" hidden="0" customHeight="1">
+      <x:c r="A20" s="19" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="B20" s="19" t="str">
+        <x:v>RF system</x:v>
+      </x:c>
+      <x:c r="C20" s="19" t="str">
+        <x:v>Antennas/cables</x:v>
+      </x:c>
+      <x:c r="D20" s="19" t="str">
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="E20" s="19" t="str">
+        <x:v>APRS and WSPR antennas/cables for onboard SMA ports</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H18" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I18" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=PCF8574N</x:v>
-      </x:c>
-      <x:c r="J18" s="19" t="str"/>
-    </x:row>
-    <x:row r="19" ht="84" hidden="0" customHeight="1">
-      <x:c r="A19" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B19" s="19" t="str">
-        <x:v>IC</x:v>
-      </x:c>
-      <x:c r="C19" s="19" t="str">
-        <x:v>U2</x:v>
-      </x:c>
-      <x:c r="D19" s="19" t="str">
-        <x:v>TC4422AVPA</x:v>
-      </x:c>
-      <x:c r="E19" s="19" t="str">
-        <x:v>MOSFET gate driver, PDIP-8</x:v>
-      </x:c>
-      <x:c r="F19" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G19" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H19" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I19" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=TC4422AVPA</x:v>
-      </x:c>
-      <x:c r="J19" s="19" t="str"/>
-    </x:row>
-    <x:row r="20" ht="120" hidden="0" customHeight="1">
-      <x:c r="A20" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B20" s="19" t="str">
-        <x:v>Battery harness</x:v>
-      </x:c>
-      <x:c r="C20" s="19" t="str">
-        <x:v>Pack holder</x:v>
-      </x:c>
-      <x:c r="D20" s="19" t="str">
-        <x:v>BH3AAW</x:v>
-      </x:c>
-      <x:c r="E20" s="19" t="str">
-        <x:v>MPD 3xAA holder, 6-inch 24 AWG leads</x:v>
-      </x:c>
-      <x:c r="F20" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="G20" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H20" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I20" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/mpd-memory-protection-devices/BH3AAW/32050</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I20" s="19" t="str"/>
       <x:c r="J20" s="19" t="str">
-        <x:v>Off-board; pulse/cold qualification required</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="96" hidden="0" customHeight="1">
+        <x:v>Needs selected bands, payload geometry, cable length, and VSWR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="120" hidden="0" customHeight="1">
       <x:c r="A21" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B21" s="19" t="str">
-        <x:v>Battery harness</x:v>
+        <x:v>Cutdown</x:v>
       </x:c>
       <x:c r="C21" s="19" t="str">
-        <x:v>J1 mate</x:v>
+        <x:v>Burn element</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
-        <x:v>PHR-2</x:v>
+        <x:v>TBD Nichrome 80</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
-        <x:v>JST PH 2-position receptacle housing</x:v>
+        <x:v>Nichrome gauge and active length</x:v>
       </x:c>
       <x:c r="F21" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H21" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I21" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/jst-sales-america-inc/PHR-2/608607</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I21" s="19" t="str"/>
       <x:c r="J21" s="19" t="str">
-        <x:v>Housing only</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="96" hidden="0" customHeight="1">
+        <x:v>Bench-select against verified LightHAB OUT1 rating and cold battery behavior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="60" hidden="0" customHeight="1">
       <x:c r="A22" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B22" s="19" t="str">
-        <x:v>Battery harness</x:v>
+        <x:v>Cutdown</x:v>
       </x:c>
       <x:c r="C22" s="19" t="str">
-        <x:v>J1 leads</x:v>
+        <x:v>Burn-wire joint</x:v>
       </x:c>
       <x:c r="D22" s="19" t="str">
-        <x:v>ASPHSPH24K152</x:v>
+        <x:v>TBD crimp sleeve</x:v>
       </x:c>
       <x:c r="E22" s="19" t="str">
-        <x:v>24 AWG 6-inch pre-crimp socket-to-socket lead</x:v>
+        <x:v>Nichrome-to-copper mechanical splice</x:v>
       </x:c>
       <x:c r="F22" s="20" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I22" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=ASPHSPH24K152</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I22" s="19" t="str"/>
       <x:c r="J22" s="19" t="str">
-        <x:v>Cut in half; permanently mark polarity</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="84" hidden="0" customHeight="1">
+        <x:v>Size after wire selection; do not rely on solder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="120" hidden="0" customHeight="1">
       <x:c r="A23" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B23" s="19" t="str">
-        <x:v>Cutdown harness</x:v>
+        <x:v>Mechanical</x:v>
       </x:c>
       <x:c r="C23" s="19" t="str">
-        <x:v>J5 mate</x:v>
+        <x:v>Flight module spacers</x:v>
       </x:c>
       <x:c r="D23" s="19" t="str">
-        <x:v>XHP-2</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E23" s="19" t="str">
-        <x:v>JST XH 2-position receptacle housing</x:v>
+        <x:v>Final LightHAB mounting hardware</x:v>
       </x:c>
       <x:c r="F23" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G23" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H23" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I23" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=XHP-2</x:v>
-      </x:c>
+        <x:v>TBD</x:v>
+      </x:c>
+      <x:c r="I23" s="19" t="str"/>
       <x:c r="J23" s="19" t="str">
-        <x:v>Housing only</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="120" hidden="0" customHeight="1">
-      <x:c r="A24" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B24" s="19" t="str">
-        <x:v>Cutdown harness</x:v>
-      </x:c>
-      <x:c r="C24" s="19" t="str">
-        <x:v>J5 leads</x:v>
-      </x:c>
-      <x:c r="D24" s="19" t="str">
-        <x:v>ASXHSXH22K152</x:v>
-      </x:c>
-      <x:c r="E24" s="19" t="str">
-        <x:v>22 AWG 6-inch pre-crimp socket-to-socket lead</x:v>
-      </x:c>
-      <x:c r="F24" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G24" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H24" s="19" t="str">
-        <x:v>DigiKey</x:v>
-      </x:c>
-      <x:c r="I24" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/jst-sales-america-inc/ASXHSXH22K152/6684931</x:v>
-      </x:c>
-      <x:c r="J24" s="19" t="str">
-        <x:v>Cut in half; identify PACK+ and FET-</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="48" hidden="0" customHeight="1">
-      <x:c r="A25" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B25" s="19" t="str">
-        <x:v>Power</x:v>
-      </x:c>
-      <x:c r="C25" s="19" t="str">
-        <x:v>Flight/test cells</x:v>
-      </x:c>
-      <x:c r="D25" s="19" t="str">
-        <x:v>Energizer L91</x:v>
-      </x:c>
-      <x:c r="E25" s="19" t="str">
-        <x:v>AA lithium primary cell</x:v>
-      </x:c>
-      <x:c r="F25" s="20" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G25" s="20" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="H25" s="19" t="str">
-        <x:v>Authorized retailer</x:v>
-      </x:c>
-      <x:c r="I25" s="19" t="str">
-        <x:v>https://data.energizer.com/pdfs/l91.pdf</x:v>
-      </x:c>
-      <x:c r="J25" s="19" t="str">
-        <x:v>Two matched 3-cell sets</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="84" hidden="0" customHeight="1">
-      <x:c r="A26" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B26" s="19" t="str">
-        <x:v>Storage</x:v>
-      </x:c>
-      <x:c r="C26" s="19" t="str">
-        <x:v>OpenLog media</x:v>
-      </x:c>
-      <x:c r="D26" s="19" t="str">
-        <x:v>microSDHC &lt;=32 GB</x:v>
-      </x:c>
-      <x:c r="E26" s="19" t="str">
-        <x:v>FAT32 microSD card</x:v>
-      </x:c>
-      <x:c r="F26" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G26" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H26" s="19" t="str">
-        <x:v>Reputable retailer</x:v>
-      </x:c>
-      <x:c r="I26" s="19" t="str">
-        <x:v>https://www.sparkfun.com/sparkfun-openlog-with-headers.html</x:v>
-      </x:c>
-      <x:c r="J26" s="19" t="str">
-        <x:v>One spare</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="48" hidden="0" customHeight="1">
-      <x:c r="A27" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B27" s="19" t="str">
-        <x:v>Mechanical fit tool</x:v>
-      </x:c>
-      <x:c r="C27" s="19" t="str">
-        <x:v>Module spacing</x:v>
-      </x:c>
-      <x:c r="D27" s="19" t="str">
-        <x:v>M2 nylon hardware assortment</x:v>
-      </x:c>
-      <x:c r="E27" s="19" t="str">
-        <x:v>M2 spacers, screws, nuts</x:v>
-      </x:c>
-      <x:c r="F27" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G27" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H27" s="19" t="str">
-        <x:v>Local supplier</x:v>
-      </x:c>
-      <x:c r="I27" s="19" t="str"/>
-      <x:c r="J27" s="19" t="str">
-        <x:v>Fit tool only; final height held</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="72" hidden="0" customHeight="1">
-      <x:c r="A28" s="19" t="str">
-        <x:v>BUY NOW</x:v>
-      </x:c>
-      <x:c r="B28" s="19" t="str">
-        <x:v>Consumable</x:v>
-      </x:c>
-      <x:c r="C28" s="19" t="str">
-        <x:v>Harness splices</x:v>
-      </x:c>
-      <x:c r="D28" s="19" t="str">
-        <x:v>22-24 AWG adhesive heat-shrink</x:v>
-      </x:c>
-      <x:c r="E28" s="19" t="str">
-        <x:v>Adhesive-lined heat-shrink assortment</x:v>
-      </x:c>
-      <x:c r="F28" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G28" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H28" s="19" t="str">
-        <x:v>Local supplier</x:v>
-      </x:c>
-      <x:c r="I28" s="19" t="str"/>
-      <x:c r="J28" s="19" t="str">
-        <x:v>Copper splice insulation only</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="72" hidden="0" customHeight="1">
-      <x:c r="A29" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B29" s="19" t="str">
-        <x:v>Fabrication</x:v>
-      </x:c>
-      <x:c r="C29" s="19" t="str">
-        <x:v>Carrier PCB</x:v>
-      </x:c>
-      <x:c r="D29" s="19" t="str">
-        <x:v>Bare PCB</x:v>
-      </x:c>
-      <x:c r="E29" s="19" t="str">
-        <x:v>Fabricated weather-balloon-logger carrier</x:v>
-      </x:c>
-      <x:c r="F29" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G29" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H29" s="19" t="str">
-        <x:v>PCB fabricator</x:v>
-      </x:c>
-      <x:c r="I29" s="19" t="str"/>
-      <x:c r="J29" s="19" t="str">
-        <x:v>Order only after exact-parts 1:1 fit gate passes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="84" hidden="0" customHeight="1">
-      <x:c r="A30" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B30" s="19" t="str">
-        <x:v>RF system</x:v>
-      </x:c>
-      <x:c r="C30" s="19" t="str">
-        <x:v>APRS</x:v>
-      </x:c>
-      <x:c r="D30" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="E30" s="19" t="str">
-        <x:v>144-146 MHz antenna and 50-ohm SMA-male cable</x:v>
-      </x:c>
-      <x:c r="F30" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G30" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H30" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I30" s="19" t="str"/>
-      <x:c r="J30" s="19" t="str">
-        <x:v>Needs payload geometry, cable length, VSWR</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="72" hidden="0" customHeight="1">
-      <x:c r="A31" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B31" s="19" t="str">
-        <x:v>RF system</x:v>
-      </x:c>
-      <x:c r="C31" s="19" t="str">
-        <x:v>WSPR</x:v>
-      </x:c>
-      <x:c r="D31" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="E31" s="19" t="str">
-        <x:v>Band-specific LPF, antenna, and SMA-male cable</x:v>
-      </x:c>
-      <x:c r="F31" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G31" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H31" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I31" s="19" t="str"/>
-      <x:c r="J31" s="19" t="str">
-        <x:v>Band is not released; onboard HF LPF absent</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="60" hidden="0" customHeight="1">
-      <x:c r="A32" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B32" s="19" t="str">
-        <x:v>Cutdown</x:v>
-      </x:c>
-      <x:c r="C32" s="19" t="str">
-        <x:v>Burn element</x:v>
-      </x:c>
-      <x:c r="D32" s="19" t="str">
-        <x:v>TBD Nichrome 80</x:v>
-      </x:c>
-      <x:c r="E32" s="19" t="str">
-        <x:v>Nichrome gauge and active length</x:v>
-      </x:c>
-      <x:c r="F32" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G32" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H32" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I32" s="19" t="str"/>
-      <x:c r="J32" s="19" t="str">
-        <x:v>Bench-select for 3.0-5.4 V, &lt;=2 A, &lt;=30 s</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="60" hidden="0" customHeight="1">
-      <x:c r="A33" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B33" s="19" t="str">
-        <x:v>Cutdown</x:v>
-      </x:c>
-      <x:c r="C33" s="19" t="str">
-        <x:v>Burn-wire joint</x:v>
-      </x:c>
-      <x:c r="D33" s="19" t="str">
-        <x:v>TBD crimp sleeve</x:v>
-      </x:c>
-      <x:c r="E33" s="19" t="str">
-        <x:v>Nichrome-to-copper mechanical splice</x:v>
-      </x:c>
-      <x:c r="F33" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G33" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H33" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I33" s="19" t="str"/>
-      <x:c r="J33" s="19" t="str">
-        <x:v>Size after wire selection; do not rely on solder</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="72" hidden="0" customHeight="1">
-      <x:c r="A34" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B34" s="19" t="str">
-        <x:v>Mechanical</x:v>
-      </x:c>
-      <x:c r="C34" s="19" t="str">
-        <x:v>Flight module spacers</x:v>
-      </x:c>
-      <x:c r="D34" s="19" t="str">
-        <x:v>TBD M2 standoffs</x:v>
-      </x:c>
-      <x:c r="E34" s="19" t="str">
-        <x:v>Final LightAPRS mounting hardware</x:v>
-      </x:c>
-      <x:c r="F34" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G34" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H34" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I34" s="19" t="str"/>
-      <x:c r="J34" s="19" t="str">
-        <x:v>Measure physical stack and hole centers first</x:v>
+        <x:v>Measure physical stack, holes, battery holder, USB, and SMA clearance first</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:A34">
+  <x:conditionalFormatting sqref="A2:A23">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="BUY NOW"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="HOLD"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69215ccbe1e046a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02af7720b016434d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1709,13 +1363,13 @@
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" s="22" t="str">
-        <x:v>Bare PCB fabrication</x:v>
+        <x:v>LightHAB J1/J2/J3 interfaces</x:v>
       </x:c>
       <x:c r="B2" s="22" t="str">
-        <x:v>Exact-parts fit gate precedes fabrication</x:v>
+        <x:v>Vendor mechanical geometry is not published</x:v>
       </x:c>
       <x:c r="C2" s="22" t="str">
-        <x:v>Place all board parts and LightAPRS on the 1:1 PDF; verify scale, bodies, holes, connector access, and cable bends</x:v>
+        <x:v>Measure pitch, hole diameter, row location, orientation, and solder access on the purchased board</x:v>
       </x:c>
       <x:c r="D2" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1723,13 +1377,13 @@
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" s="22" t="str">
-        <x:v>APRS antenna/cable</x:v>
+        <x:v>LightHAB mounting holes</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>Payload geometry and cable length not released</x:v>
+        <x:v>Provisional carrier coordinates are not authoritative</x:v>
       </x:c>
       <x:c r="C3" s="22" t="str">
-        <x:v>Select enclosure layout and verify 50-ohm SMA-male mate plus VHF VSWR</x:v>
+        <x:v>Measure all centers and diameters; update H1-H4 and the module outline</x:v>
       </x:c>
       <x:c r="D3" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1737,13 +1391,13 @@
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" s="22" t="str">
-        <x:v>WSPR LPF/antenna/cable</x:v>
+        <x:v>Bare PCB fabrication</x:v>
       </x:c>
       <x:c r="B4" s="22" t="str">
-        <x:v>Band not released; module has no onboard HF LPF</x:v>
+        <x:v>Measured-module fit gate precedes fabrication</x:v>
       </x:c>
       <x:c r="C4" s="22" t="str">
-        <x:v>Select authorized band; design filter/antenna; verify match and harmonics</x:v>
+        <x:v>Update CAD, print the 1:1 PDF, and verify all exact parts plus USB/SMA/battery clearances</x:v>
       </x:c>
       <x:c r="D4" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1751,13 +1405,13 @@
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" s="22" t="str">
-        <x:v>Nichrome wire</x:v>
+        <x:v>APRS/WSPR antennas and cables</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
-        <x:v>Gauge/length set resistance and current</x:v>
+        <x:v>Bands and payload geometry are not released</x:v>
       </x:c>
       <x:c r="C5" s="22" t="str">
-        <x:v>Cold bench test from 3.0-5.4 V within &lt;=2 A and &lt;=30 s</x:v>
+        <x:v>Select bands and enclosure layout; verify SMA mating, cable routing, match, and harmonics</x:v>
       </x:c>
       <x:c r="D5" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1765,13 +1419,13 @@
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="22" t="str">
-        <x:v>Nichrome sleeves</x:v>
+        <x:v>Nichrome wire</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>Sleeve size follows final wire diameters</x:v>
+        <x:v>Gauge/length set resistance and current</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
-        <x:v>Choose compatible mechanical crimps; prove pull strength and contact heating</x:v>
+        <x:v>Verify LightHAB OUT1 rating, then cold-test the selected wire and pulse duration</x:v>
       </x:c>
       <x:c r="D6" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1779,22 +1433,50 @@
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" s="22" t="str">
-        <x:v>Final M2 spacers</x:v>
+        <x:v>Nichrome sleeves</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
+        <x:v>Sleeve size follows final wire diameters</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>Choose compatible mechanical crimps; prove pull strength and contact heating</x:v>
+      </x:c>
+      <x:c r="D7" s="25" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="22" t="str">
+        <x:v>Final mounting hardware</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
         <x:v>Physical module stack-up remains unmeasured</x:v>
       </x:c>
-      <x:c r="C7" s="22" t="str">
-        <x:v>Measure hole centers and clearance; select exact spacer length/material</x:v>
-      </x:c>
-      <x:c r="D7" s="25" t="str">
+      <x:c r="C8" s="22" t="str">
+        <x:v>Measure hole diameter, board spacing, battery holder, USB, SMA, and underside clearance</x:v>
+      </x:c>
+      <x:c r="D8" s="25" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="22" t="str">
+        <x:v>LightHAB VBATT/OUT1 behavior</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>Switch routing and pyro current rating are unverified</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>Bench-confirm switched VBATT and qualify OUT1 with an inert load before attaching nichrome</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
         <x:v>OPEN</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf580ccb248564154"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ea044d038ce43e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(power): use LightHAB 3V3 for OpenLog
Remove the separate VBATT-fed regulator path. Keep host rail capacity as a bench-test gate before fabrication.
</commit_message>
<xml_diff>
--- a/outputs/fit-check-order-list.xlsx
+++ b/outputs/fit-check-order-list.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1638369846bf4564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order List" sheetId="2" r:id="R3a8c42fd0a8d46d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hold Closure" sheetId="3" r:id="Re447713810184260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc161c176485b4707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order List" sheetId="2" r:id="R1772f9a41d984dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hold Closure" sheetId="3" r:id="Re9372ce6750b4281"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,8 +212,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FitCheckOrderTable" displayName="FitCheckOrderTable" ref="A1:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:J23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FitCheckOrderTable" displayName="FitCheckOrderTable" ref="A1:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J21"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Status"/>
     <x:tableColumn id="2" name="Category"/>
@@ -460,7 +460,7 @@
         <x:v>Prepared</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-22</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -476,8 +476,8 @@
         <x:v>Buy-now line items</x:v>
       </x:c>
       <x:c r="B5" s="9" t="n">
-        <x:f>COUNTIF('Order List'!$A$2:$A$23,"BUY NOW")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Order List'!$A$2:$A$21,"BUY NOW")</x:f>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -485,8 +485,8 @@
         <x:v>Held line items</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:f>COUNTIF('Order List'!$A$2:$A$23,"HOLD")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Order List'!$A$2:$A$21,"HOLD")</x:f>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -494,7 +494,7 @@
         <x:v>Required populated PCB refs</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -538,7 +538,7 @@
         <x:v>Measure LightHAB first</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>J1/J2/J3 and all four mounting holes remain provisional until the purchased tracker is measured.</x:v>
+        <x:v>J2/J3 and all four mounting holes remain provisional until the purchased tracker is measured.</x:v>
       </x:c>
       <x:c r="D12" s="12"/>
       <x:c r="E12" s="12"/>
@@ -675,7 +675,7 @@
         <x:v>Exact with-headers version</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="48" hidden="0" customHeight="1">
+    <x:row r="3" ht="84" hidden="0" customHeight="1">
       <x:c r="A3" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
@@ -683,13 +683,13 @@
         <x:v>Module</x:v>
       </x:c>
       <x:c r="C3" s="19" t="str">
-        <x:v>A2</x:v>
+        <x:v>Host</x:v>
       </x:c>
       <x:c r="D3" s="19" t="str">
-        <x:v>2123</x:v>
+        <x:v>LightHABTracker 1.0</x:v>
       </x:c>
       <x:c r="E3" s="19" t="str">
-        <x:v>Pololu S7V8F5 fixed 5 V regulator</x:v>
+        <x:v>GPS/APRS/WSPR tracker with 3xAA holder and two pyro outputs</x:v>
       </x:c>
       <x:c r="F3" s="20" t="n">
         <x:v>1</x:v>
@@ -698,45 +698,45 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H3" s="19" t="str">
-        <x:v>Pololu</x:v>
+        <x:v>QRP Labs</x:v>
       </x:c>
       <x:c r="I3" s="19" t="str">
-        <x:v>https://www.pololu.com/product/2123</x:v>
+        <x:v>https://shop.qrp-labs.com/aprs/LightHABTracker</x:v>
       </x:c>
       <x:c r="J3" s="19" t="str">
-        <x:v>Use included straight header</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="84" hidden="0" customHeight="1">
+        <x:v>Measure the purchased board before fabricating the carrier</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="96" hidden="0" customHeight="1">
       <x:c r="A4" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B4" s="19" t="str">
-        <x:v>Module</x:v>
+        <x:v>Capacitor</x:v>
       </x:c>
       <x:c r="C4" s="19" t="str">
-        <x:v>Host</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="D4" s="19" t="str">
-        <x:v>LightHABTracker 1.0</x:v>
+        <x:v>C322C475K5R5TA</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>GPS/APRS/WSPR tracker with 3xAA holder and two pyro outputs</x:v>
+        <x:v>4.7 uF radial THT capacitor</x:v>
       </x:c>
       <x:c r="F4" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H4" s="19" t="str">
-        <x:v>QRP Labs</x:v>
+        <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I4" s="19" t="str">
-        <x:v>https://shop.qrp-labs.com/aprs/LightHABTracker</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=C322C475K5R5TA</x:v>
       </x:c>
       <x:c r="J4" s="19" t="str">
-        <x:v>Measure the purchased board before fabricating the carrier</x:v>
+        <x:v>Prototype spares included</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="96" hidden="0" customHeight="1">
@@ -747,77 +747,75 @@
         <x:v>Capacitor</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>C1</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>C322C475K5R5TA</x:v>
+        <x:v>C315C104K5R5TA</x:v>
       </x:c>
       <x:c r="E5" s="19" t="str">
-        <x:v>4.7 uF radial THT capacitor</x:v>
+        <x:v>0.1 uF radial THT capacitor</x:v>
       </x:c>
       <x:c r="F5" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="20" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H5" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I5" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=C322C475K5R5TA</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=C315C104K5R5TA</x:v>
       </x:c>
       <x:c r="J5" s="19" t="str">
         <x:v>Prototype spares included</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="96" hidden="0" customHeight="1">
+    <x:row r="6" ht="84" hidden="0" customHeight="1">
       <x:c r="A6" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
-        <x:v>Capacitor</x:v>
+        <x:v>LED</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>C2</x:v>
+        <x:v>D1</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
-        <x:v>C315C104K5R5TA</x:v>
+        <x:v>WP710A10SGC</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>0.1 uF radial THT capacitor</x:v>
+        <x:v>3 mm green THT LED</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="20" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H6" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I6" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=C315C104K5R5TA</x:v>
-      </x:c>
-      <x:c r="J6" s="19" t="str">
-        <x:v>Prototype spares included</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="84" hidden="0" customHeight="1">
+        <x:v>https://www.digikey.com/en/products/result?keywords=WP710A10SGC</x:v>
+      </x:c>
+      <x:c r="J6" s="19" t="str"/>
+    </x:row>
+    <x:row r="7" ht="108" hidden="0" customHeight="1">
       <x:c r="A7" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
-        <x:v>LED</x:v>
+        <x:v>PCB connector</x:v>
       </x:c>
       <x:c r="C7" s="19" t="str">
-        <x:v>D1</x:v>
+        <x:v>J5</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
-        <x:v>WP710A10SGC</x:v>
+        <x:v>S2B-XH-A(LF)(SN)</x:v>
       </x:c>
       <x:c r="E7" s="19" t="str">
-        <x:v>3 mm green THT LED</x:v>
+        <x:v>JST XH 2-pin side-entry THT header</x:v>
       </x:c>
       <x:c r="F7" s="20" t="n">
         <x:v>1</x:v>
@@ -829,41 +827,41 @@
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I7" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=WP710A10SGC</x:v>
-      </x:c>
-      <x:c r="J7" s="19" t="str"/>
-    </x:row>
-    <x:row r="8" ht="108" hidden="0" customHeight="1">
+        <x:v>https://www.digikey.com/en/products/result?keywords=S2B-XH-A%28LF%29%28SN%29</x:v>
+      </x:c>
+      <x:c r="J7" s="19" t="str">
+        <x:v>Cutdown output</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="96" hidden="0" customHeight="1">
       <x:c r="A8" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B8" s="19" t="str">
-        <x:v>PCB connector</x:v>
+        <x:v>Resistor</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
-        <x:v>J5</x:v>
+        <x:v>R1,R4</x:v>
       </x:c>
       <x:c r="D8" s="19" t="str">
-        <x:v>S2B-XH-A(LF)(SN)</x:v>
+        <x:v>MFR-25FBF52-1K</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>JST XH 2-pin side-entry THT header</x:v>
+        <x:v>1 kohm 1% 1/4 W axial</x:v>
       </x:c>
       <x:c r="F8" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G8" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I8" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=S2B-XH-A%28LF%29%28SN%29</x:v>
-      </x:c>
-      <x:c r="J8" s="19" t="str">
-        <x:v>Cutdown output</x:v>
-      </x:c>
+        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-1K/13011</x:v>
+      </x:c>
+      <x:c r="J8" s="19" t="str"/>
     </x:row>
     <x:row r="9" ht="96" hidden="0" customHeight="1">
       <x:c r="A9" s="19" t="str">
@@ -873,61 +871,63 @@
         <x:v>Resistor</x:v>
       </x:c>
       <x:c r="C9" s="19" t="str">
-        <x:v>R1,R4</x:v>
+        <x:v>R2</x:v>
       </x:c>
       <x:c r="D9" s="19" t="str">
-        <x:v>MFR-25FBF52-1K</x:v>
+        <x:v>MFR-25FBF52-100K</x:v>
       </x:c>
       <x:c r="E9" s="19" t="str">
-        <x:v>1 kohm 1% 1/4 W axial</x:v>
+        <x:v>100 kohm 1% 1/4 W axial</x:v>
       </x:c>
       <x:c r="F9" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="20" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H9" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I9" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/yageo/MFR-25FBF52-1K/13011</x:v>
-      </x:c>
-      <x:c r="J9" s="19" t="str"/>
-    </x:row>
-    <x:row r="10" ht="96" hidden="0" customHeight="1">
+        <x:v>https://www.digikey.com/en/products/result?keywords=MFR-25FBF52-100K</x:v>
+      </x:c>
+      <x:c r="J9" s="19" t="str">
+        <x:v>LED reset-default-off pull-up</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="84" hidden="0" customHeight="1">
       <x:c r="A10" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B10" s="19" t="str">
-        <x:v>Resistor</x:v>
+        <x:v>Cutdown harness</x:v>
       </x:c>
       <x:c r="C10" s="19" t="str">
-        <x:v>R2</x:v>
+        <x:v>J5 mate</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>MFR-25FBF52-100K</x:v>
+        <x:v>XHP-2</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>100 kohm 1% 1/4 W axial</x:v>
+        <x:v>JST XH 2-position receptacle housing</x:v>
       </x:c>
       <x:c r="F10" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="20" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H10" s="19" t="str">
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I10" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=MFR-25FBF52-100K</x:v>
+        <x:v>https://www.digikey.com/en/products/result?keywords=XHP-2</x:v>
       </x:c>
       <x:c r="J10" s="19" t="str">
-        <x:v>LED reset-default-off pull-up</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="84" hidden="0" customHeight="1">
+        <x:v>Housing only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="120" hidden="0" customHeight="1">
       <x:c r="A11" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
@@ -935,16 +935,16 @@
         <x:v>Cutdown harness</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
-        <x:v>J5 mate</x:v>
+        <x:v>J5 leads</x:v>
       </x:c>
       <x:c r="D11" s="19" t="str">
-        <x:v>XHP-2</x:v>
+        <x:v>ASXHSXH22K152</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:v>JST XH 2-position receptacle housing</x:v>
+        <x:v>22 AWG 6-inch pre-crimp socket-to-socket lead</x:v>
       </x:c>
       <x:c r="F11" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="20" t="n">
         <x:v>2</x:v>
@@ -953,136 +953,134 @@
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="I11" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/result?keywords=XHP-2</x:v>
+        <x:v>https://www.digikey.com/en/products/detail/jst-sales-america-inc/ASXHSXH22K152/6684931</x:v>
       </x:c>
       <x:c r="J11" s="19" t="str">
-        <x:v>Housing only</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="120" hidden="0" customHeight="1">
+        <x:v>Cut in half; identify OUT1 and GND</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" hidden="0" customHeight="1">
       <x:c r="A12" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B12" s="19" t="str">
-        <x:v>Cutdown harness</x:v>
+        <x:v>Power</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>J5 leads</x:v>
+        <x:v>Flight/test cells</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>ASXHSXH22K152</x:v>
+        <x:v>Energizer L91</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>22 AWG 6-inch pre-crimp socket-to-socket lead</x:v>
+        <x:v>AA lithium primary cell</x:v>
       </x:c>
       <x:c r="F12" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G12" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>DigiKey</x:v>
+        <x:v>Authorized retailer</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>https://www.digikey.com/en/products/detail/jst-sales-america-inc/ASXHSXH22K152/6684931</x:v>
+        <x:v>https://data.energizer.com/pdfs/l91.pdf</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>Cut in half; identify PACK+ and FET-</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" hidden="0" customHeight="1">
+        <x:v>Two matched 3-cell sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="84" hidden="0" customHeight="1">
       <x:c r="A13" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
-        <x:v>Power</x:v>
+        <x:v>Storage</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:v>Flight/test cells</x:v>
+        <x:v>OpenLog media</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str">
-        <x:v>Energizer L91</x:v>
+        <x:v>microSDHC &lt;=32 GB</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:v>AA lithium primary cell</x:v>
+        <x:v>FAT32 microSD card</x:v>
       </x:c>
       <x:c r="F13" s="20" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="20" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
-        <x:v>Authorized retailer</x:v>
+        <x:v>Reputable retailer</x:v>
       </x:c>
       <x:c r="I13" s="19" t="str">
-        <x:v>https://data.energizer.com/pdfs/l91.pdf</x:v>
+        <x:v>https://www.sparkfun.com/sparkfun-openlog-with-headers.html</x:v>
       </x:c>
       <x:c r="J13" s="19" t="str">
-        <x:v>Two matched 3-cell sets</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="84" hidden="0" customHeight="1">
+        <x:v>One spare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="60" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="str">
         <x:v>BUY NOW</x:v>
       </x:c>
       <x:c r="B14" s="19" t="str">
-        <x:v>Storage</x:v>
+        <x:v>Mechanical fit tool</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>OpenLog media</x:v>
+        <x:v>Module spacing</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str">
-        <x:v>microSDHC &lt;=32 GB</x:v>
+        <x:v>M2/M2.5 nylon hardware assortment</x:v>
       </x:c>
       <x:c r="E14" s="19" t="str">
-        <x:v>FAT32 microSD card</x:v>
+        <x:v>Spacers, screws, and nuts</x:v>
       </x:c>
       <x:c r="F14" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G14" s="20" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H14" s="19" t="str">
-        <x:v>Reputable retailer</x:v>
-      </x:c>
-      <x:c r="I14" s="19" t="str">
-        <x:v>https://www.sparkfun.com/sparkfun-openlog-with-headers.html</x:v>
-      </x:c>
+        <x:v>Local supplier</x:v>
+      </x:c>
+      <x:c r="I14" s="19" t="str"/>
       <x:c r="J14" s="19" t="str">
-        <x:v>One spare</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="60" hidden="0" customHeight="1">
+        <x:v>Fit tool only; final diameter and height held</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="96" hidden="0" customHeight="1">
       <x:c r="A15" s="19" t="str">
-        <x:v>BUY NOW</x:v>
+        <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B15" s="19" t="str">
-        <x:v>Mechanical fit tool</x:v>
+        <x:v>Module interface</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:v>Module spacing</x:v>
+        <x:v>J2</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
-        <x:v>M2/M2.5 nylon hardware assortment</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
-        <x:v>Spacers, screws, and nuts</x:v>
+        <x:v>Nine-position signal solder interface</x:v>
       </x:c>
       <x:c r="F15" s="20" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
-        <x:v>Local supplier</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="I15" s="19" t="str"/>
       <x:c r="J15" s="19" t="str">
-        <x:v>Fit tool only; final diameter and height held</x:v>
+        <x:v>Verify actual row pitch, location, and installed header direction</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="84" hidden="0" customHeight="1">
@@ -1093,13 +1091,13 @@
         <x:v>Module interface</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>J1</x:v>
+        <x:v>J3</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str">
         <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E16" s="19" t="str">
-        <x:v>Two-position VBATT/GND solder interface</x:v>
+        <x:v>Two-position OUT1/GND solder interface</x:v>
       </x:c>
       <x:c r="F16" s="20" t="n">
         <x:v>1</x:v>
@@ -1115,21 +1113,21 @@
         <x:v>Measure pad pitch, hole size, and mating method on LightHAB</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="96" hidden="0" customHeight="1">
+    <x:row r="17" ht="72" hidden="0" customHeight="1">
       <x:c r="A17" s="19" t="str">
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B17" s="19" t="str">
-        <x:v>Module interface</x:v>
+        <x:v>Fabrication</x:v>
       </x:c>
       <x:c r="C17" s="19" t="str">
-        <x:v>J2</x:v>
+        <x:v>Carrier PCB</x:v>
       </x:c>
       <x:c r="D17" s="19" t="str">
-        <x:v>TBD after measurement</x:v>
+        <x:v>Bare PCB</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
-        <x:v>Nine-position signal solder interface</x:v>
+        <x:v>Fabricated weather-balloon-logger carrier</x:v>
       </x:c>
       <x:c r="F17" s="20" t="n">
         <x:v>1</x:v>
@@ -1138,31 +1136,31 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>PCB fabricator</x:v>
       </x:c>
       <x:c r="I17" s="19" t="str"/>
       <x:c r="J17" s="19" t="str">
-        <x:v>Verify actual row pitch, location, and installed header direction</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="84" hidden="0" customHeight="1">
+        <x:v>Order only after exact-parts 1:1 fit gate passes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="108" hidden="0" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B18" s="19" t="str">
-        <x:v>Module interface</x:v>
+        <x:v>RF system</x:v>
       </x:c>
       <x:c r="C18" s="19" t="str">
-        <x:v>J3</x:v>
+        <x:v>Antennas/cables</x:v>
       </x:c>
       <x:c r="D18" s="19" t="str">
-        <x:v>TBD after measurement</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="E18" s="19" t="str">
-        <x:v>Two-position OUT1/GND solder interface</x:v>
+        <x:v>APRS and WSPR antennas/cables for onboard SMA ports</x:v>
       </x:c>
       <x:c r="F18" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="20" t="n">
         <x:v>0</x:v>
@@ -1172,24 +1170,24 @@
       </x:c>
       <x:c r="I18" s="19" t="str"/>
       <x:c r="J18" s="19" t="str">
-        <x:v>Measure pad pitch, hole size, and mating method on LightHAB</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="72" hidden="0" customHeight="1">
+        <x:v>Needs selected bands, payload geometry, cable length, and VSWR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="120" hidden="0" customHeight="1">
       <x:c r="A19" s="19" t="str">
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B19" s="19" t="str">
-        <x:v>Fabrication</x:v>
+        <x:v>Cutdown</x:v>
       </x:c>
       <x:c r="C19" s="19" t="str">
-        <x:v>Carrier PCB</x:v>
+        <x:v>Burn element</x:v>
       </x:c>
       <x:c r="D19" s="19" t="str">
-        <x:v>Bare PCB</x:v>
+        <x:v>TBD Nichrome 80</x:v>
       </x:c>
       <x:c r="E19" s="19" t="str">
-        <x:v>Fabricated weather-balloon-logger carrier</x:v>
+        <x:v>Nichrome gauge and active length</x:v>
       </x:c>
       <x:c r="F19" s="20" t="n">
         <x:v>1</x:v>
@@ -1198,28 +1196,28 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="H19" s="19" t="str">
-        <x:v>PCB fabricator</x:v>
+        <x:v>TBD</x:v>
       </x:c>
       <x:c r="I19" s="19" t="str"/>
       <x:c r="J19" s="19" t="str">
-        <x:v>Order only after exact-parts 1:1 fit gate passes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="108" hidden="0" customHeight="1">
+        <x:v>Bench-select against verified LightHAB OUT1 rating and cold battery behavior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="60" hidden="0" customHeight="1">
       <x:c r="A20" s="19" t="str">
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B20" s="19" t="str">
-        <x:v>RF system</x:v>
+        <x:v>Cutdown</x:v>
       </x:c>
       <x:c r="C20" s="19" t="str">
-        <x:v>Antennas/cables</x:v>
+        <x:v>Burn-wire joint</x:v>
       </x:c>
       <x:c r="D20" s="19" t="str">
-        <x:v>TBD</x:v>
+        <x:v>TBD crimp sleeve</x:v>
       </x:c>
       <x:c r="E20" s="19" t="str">
-        <x:v>APRS and WSPR antennas/cables for onboard SMA ports</x:v>
+        <x:v>Nichrome-to-copper mechanical splice</x:v>
       </x:c>
       <x:c r="F20" s="20" t="n">
         <x:v>2</x:v>
@@ -1232,7 +1230,7 @@
       </x:c>
       <x:c r="I20" s="19" t="str"/>
       <x:c r="J20" s="19" t="str">
-        <x:v>Needs selected bands, payload geometry, cable length, and VSWR</x:v>
+        <x:v>Size after wire selection; do not rely on solder</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="120" hidden="0" customHeight="1">
@@ -1240,19 +1238,19 @@
         <x:v>HOLD</x:v>
       </x:c>
       <x:c r="B21" s="19" t="str">
-        <x:v>Cutdown</x:v>
+        <x:v>Mechanical</x:v>
       </x:c>
       <x:c r="C21" s="19" t="str">
-        <x:v>Burn element</x:v>
+        <x:v>Flight module spacers</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
-        <x:v>TBD Nichrome 80</x:v>
+        <x:v>TBD after measurement</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
-        <x:v>Nichrome gauge and active length</x:v>
+        <x:v>Final LightHAB mounting hardware</x:v>
       </x:c>
       <x:c r="F21" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="20" t="n">
         <x:v>0</x:v>
@@ -1262,77 +1260,17 @@
       </x:c>
       <x:c r="I21" s="19" t="str"/>
       <x:c r="J21" s="19" t="str">
-        <x:v>Bench-select against verified LightHAB OUT1 rating and cold battery behavior</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="60" hidden="0" customHeight="1">
-      <x:c r="A22" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B22" s="19" t="str">
-        <x:v>Cutdown</x:v>
-      </x:c>
-      <x:c r="C22" s="19" t="str">
-        <x:v>Burn-wire joint</x:v>
-      </x:c>
-      <x:c r="D22" s="19" t="str">
-        <x:v>TBD crimp sleeve</x:v>
-      </x:c>
-      <x:c r="E22" s="19" t="str">
-        <x:v>Nichrome-to-copper mechanical splice</x:v>
-      </x:c>
-      <x:c r="F22" s="20" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G22" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H22" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I22" s="19" t="str"/>
-      <x:c r="J22" s="19" t="str">
-        <x:v>Size after wire selection; do not rely on solder</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="120" hidden="0" customHeight="1">
-      <x:c r="A23" s="19" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="B23" s="19" t="str">
-        <x:v>Mechanical</x:v>
-      </x:c>
-      <x:c r="C23" s="19" t="str">
-        <x:v>Flight module spacers</x:v>
-      </x:c>
-      <x:c r="D23" s="19" t="str">
-        <x:v>TBD after measurement</x:v>
-      </x:c>
-      <x:c r="E23" s="19" t="str">
-        <x:v>Final LightHAB mounting hardware</x:v>
-      </x:c>
-      <x:c r="F23" s="20" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G23" s="20" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H23" s="19" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="I23" s="19" t="str"/>
-      <x:c r="J23" s="19" t="str">
         <x:v>Measure physical stack, holes, battery holder, USB, and SMA clearance first</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:A23">
+  <x:conditionalFormatting sqref="A2:A21">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="BUY NOW"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="HOLD"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02af7720b016434d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R625c3c30c81e4cd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1363,7 +1301,7 @@
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" s="22" t="str">
-        <x:v>LightHAB J1/J2/J3 interfaces</x:v>
+        <x:v>LightHAB J2/J3 interfaces</x:v>
       </x:c>
       <x:c r="B2" s="22" t="str">
         <x:v>Vendor mechanical geometry is not published</x:v>
@@ -1461,13 +1399,13 @@
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="22" t="str">
-        <x:v>LightHAB VBATT/OUT1 behavior</x:v>
+        <x:v>LightHAB 3V3/OUT1 behavior</x:v>
       </x:c>
       <x:c r="B9" s="22" t="str">
-        <x:v>Switch routing and pyro current rating are unverified</x:v>
+        <x:v>3V3 rail capacity and pyro current rating are unverified</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>Bench-confirm switched VBATT and qualify OUT1 with an inert load before attaching nichrome</x:v>
+        <x:v>Stress the 3V3 rail with OpenLog and radio activity; qualify OUT1 with an inert load before attaching nichrome</x:v>
       </x:c>
       <x:c r="D9" s="25" t="str">
         <x:v>OPEN</x:v>
@@ -1476,7 +1414,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ea044d038ce43e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47a17a995ca74736"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>